<commit_message>
Add indicator engine and Argentina structure layouts
</commit_message>
<xml_diff>
--- a/outputs/harmonized_excels/brasil.xlsx
+++ b/outputs/harmonized_excels/brasil.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/06923e1dbd627e79/repos/UNGS_informalidad_comparada/outputs/harmonized_excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_C7FB8E5BCB978FDEB73DAABA4AE38691A3082A6F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D72B603B-189B-4EAA-BC15-B4A07792F9F2}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_C7FB8E5B6C97027F999E6A1B52FF4616ACD62DF4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30010CEC-C358-452E-A373-1D571C6AC158}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="20390" yWindow="1190" windowWidth="14400" windowHeight="7310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -109,17 +109,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,18 +135,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -459,13 +446,7 @@
   <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="17" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="13.109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -475,49 +456,49 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -525,106 +506,106 @@
       <c r="A2">
         <v>2018</v>
       </c>
-      <c r="B2" s="1">
-        <v>254324</v>
+      <c r="B2">
+        <v>1611522</v>
       </c>
       <c r="C2" s="1">
-        <v>63810440</v>
+        <v>703896832</v>
       </c>
       <c r="D2" s="1">
-        <v>4104348</v>
+        <v>319961568</v>
       </c>
       <c r="E2" s="1">
-        <v>4095651.75</v>
+        <v>46496548</v>
       </c>
       <c r="F2" s="1">
-        <v>47894776</v>
+        <v>337438688</v>
       </c>
       <c r="G2" s="1">
-        <v>39063308</v>
+        <v>225133952</v>
       </c>
       <c r="H2" s="1">
-        <v>4440336.5</v>
+        <v>74769952</v>
       </c>
       <c r="I2" s="1">
-        <v>19013776</v>
+        <v>111503208</v>
       </c>
       <c r="J2" s="1">
-        <v>44796660</v>
-      </c>
-      <c r="K2" s="2">
-        <v>6.4320948108177914E-2</v>
-      </c>
-      <c r="L2" s="2">
-        <v>6.4184665550025985E-2</v>
-      </c>
-      <c r="M2" s="2">
-        <v>0.75057899616426405</v>
-      </c>
-      <c r="N2" s="2">
-        <v>0.61217738037850855</v>
-      </c>
-      <c r="O2" s="2">
-        <v>6.958636392414784E-2</v>
-      </c>
-      <c r="P2" s="2">
-        <v>0.29797280821132088</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>0.70202712910301202</v>
+        <v>208458384</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0.45455747696844301</v>
+      </c>
+      <c r="L2" s="1">
+        <v>6.6055913148363191E-2</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.47938657010463709</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0.3198394164672132</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0.1062228846627342</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0.15840845267506479</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0.29614905838928401</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2023</v>
       </c>
-      <c r="B3" s="1">
-        <v>254229</v>
+      <c r="B3">
+        <v>1393606</v>
       </c>
       <c r="C3" s="1">
-        <v>80460400</v>
+        <v>733761975.49653554</v>
       </c>
       <c r="D3" s="1">
-        <v>5578560.5</v>
+        <v>348768488.04017317</v>
       </c>
       <c r="E3" s="1">
-        <v>5598974</v>
+        <v>31089236.591390621</v>
       </c>
       <c r="F3" s="1">
-        <v>58002476</v>
+        <v>353904250.86497158</v>
       </c>
       <c r="G3" s="1">
-        <v>46020008</v>
+        <v>246634748.44859391</v>
       </c>
       <c r="H3" s="1">
-        <v>6091510</v>
+        <v>83922993.932008907</v>
       </c>
       <c r="I3" s="1">
-        <v>22833902</v>
+        <v>124742367.8845676</v>
       </c>
       <c r="J3" s="1">
-        <v>57626496</v>
-      </c>
-      <c r="K3" s="2">
-        <v>6.9332994864554492E-2</v>
-      </c>
-      <c r="L3" s="2">
-        <v>6.9586703521235291E-2</v>
-      </c>
-      <c r="M3" s="2">
-        <v>0.72088227252163795</v>
-      </c>
-      <c r="N3" s="2">
-        <v>0.57195847895362195</v>
-      </c>
-      <c r="O3" s="2">
-        <v>7.5708174456005681E-2</v>
-      </c>
-      <c r="P3" s="2">
-        <v>0.28379056032532768</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>0.71620941481772404</v>
+        <v>224026120.15560561</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.47531556511110051</v>
+      </c>
+      <c r="L3" s="1">
+        <v>4.2369647964317837E-2</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0.48231478692458157</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.33612364320418281</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0.11437359352836229</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0.1700038596305766</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0.30531170548052378</v>
       </c>
     </row>
   </sheetData>
@@ -637,7 +618,8 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -656,10 +638,10 @@
         <v>20</v>
       </c>
       <c r="B2" s="1">
-        <v>4104348</v>
+        <v>319961568</v>
       </c>
       <c r="C2" s="1">
-        <v>16112</v>
+        <v>709467</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -667,10 +649,10 @@
         <v>21</v>
       </c>
       <c r="B3" s="1">
-        <v>4095651.75</v>
+        <v>46496548</v>
       </c>
       <c r="C3" s="1">
-        <v>16958</v>
+        <v>100444</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -678,10 +660,10 @@
         <v>22</v>
       </c>
       <c r="B4" s="1">
-        <v>47894776</v>
+        <v>337438688</v>
       </c>
       <c r="C4" s="1">
-        <v>186830</v>
+        <v>801611</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -689,10 +671,10 @@
         <v>23</v>
       </c>
       <c r="B5" s="1">
-        <v>39063308</v>
+        <v>225133952</v>
       </c>
       <c r="C5" s="1">
-        <v>147555</v>
+        <v>489979</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -700,10 +682,10 @@
         <v>24</v>
       </c>
       <c r="B6" s="1">
-        <v>4440336.5</v>
+        <v>74769952</v>
       </c>
       <c r="C6" s="1">
-        <v>18196</v>
+        <v>174175</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -711,10 +693,10 @@
         <v>25</v>
       </c>
       <c r="B7" s="1">
-        <v>19013776</v>
+        <v>111503208</v>
       </c>
       <c r="C7" s="1">
-        <v>72535</v>
+        <v>262644</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -722,10 +704,10 @@
         <v>26</v>
       </c>
       <c r="B8" s="1">
-        <v>44796660</v>
+        <v>208458384</v>
       </c>
       <c r="C8" s="1">
-        <v>181789</v>
+        <v>446823</v>
       </c>
     </row>
   </sheetData>
@@ -738,7 +720,8 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -756,77 +739,77 @@
       <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="1">
-        <v>5578560.5</v>
-      </c>
-      <c r="C2" s="1">
-        <v>17750</v>
+      <c r="B2">
+        <v>348768488.04017317</v>
+      </c>
+      <c r="C2">
+        <v>630722</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="1">
-        <v>5598974</v>
-      </c>
-      <c r="C3" s="1">
-        <v>18226</v>
+      <c r="B3">
+        <v>31089236.591390621</v>
+      </c>
+      <c r="C3">
+        <v>55112</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="1">
-        <v>58002476</v>
-      </c>
-      <c r="C4" s="1">
-        <v>176456</v>
+      <c r="B4">
+        <v>353904250.86497158</v>
+      </c>
+      <c r="C4">
+        <v>707772</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="1">
-        <v>46020008</v>
-      </c>
-      <c r="C5" s="1">
-        <v>136140</v>
+      <c r="B5">
+        <v>246634748.44859391</v>
+      </c>
+      <c r="C5">
+        <v>439141</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1">
-        <v>6091510</v>
-      </c>
-      <c r="C6" s="1">
-        <v>19554</v>
+      <c r="B6">
+        <v>83922993.932008907</v>
+      </c>
+      <c r="C6">
+        <v>157303</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="1">
-        <v>22833902</v>
-      </c>
-      <c r="C7" s="1">
-        <v>68903</v>
+      <c r="B7">
+        <v>124742367.8845676</v>
+      </c>
+      <c r="C7">
+        <v>238856</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="1">
-        <v>57626496</v>
-      </c>
-      <c r="C8" s="1">
-        <v>185326</v>
+      <c r="B8">
+        <v>224026120.15560561</v>
+      </c>
+      <c r="C8">
+        <v>391866</v>
       </c>
     </row>
   </sheetData>

</xml_diff>